<commit_message>
added weight comparison to Raymer
</commit_message>
<xml_diff>
--- a/USE_THIS_DESIGN_CODE/Input Excel Sheets/Design Configurations/ZW_Snr_Proj_Initial_Design_Config.xlsx
+++ b/USE_THIS_DESIGN_CODE/Input Excel Sheets/Design Configurations/ZW_Snr_Proj_Initial_Design_Config.xlsx
@@ -4222,10 +4222,10 @@
         <v>0</v>
       </c>
       <c r="T8" s="22">
-        <v>0</v>
+        <v>7.3</v>
       </c>
       <c r="U8" s="22">
-        <v>0</v>
+        <v>1.9735</v>
       </c>
       <c r="V8" s="22">
         <v>1.0252624699999999</v>

</xml_diff>

<commit_message>
edited plots and added more fidelittyy to weigt model
</commit_message>
<xml_diff>
--- a/USE_THIS_DESIGN_CODE/Input Excel Sheets/Design Configurations/ZW_Snr_Proj_Initial_Design_Config.xlsx
+++ b/USE_THIS_DESIGN_CODE/Input Excel Sheets/Design Configurations/ZW_Snr_Proj_Initial_Design_Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10817"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14141415-9AEE-B040-8F61-03D38D173453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1252D254-2D4E-0342-873F-A1C53BC2D48F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16220" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -343,7 +343,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="274">
   <si>
     <t>Worksheet</t>
   </si>
@@ -870,9 +870,6 @@
     <t>SkinThick_v2</t>
   </si>
   <si>
-    <t>Electric</t>
-  </si>
-  <si>
     <t>Homebuilt_Composite_Prop</t>
   </si>
   <si>
@@ -999,78 +996,33 @@
     <t>W_nose</t>
   </si>
   <si>
-    <t>Xcg_nose</t>
-  </si>
-  <si>
     <t>W_fuse</t>
   </si>
   <si>
-    <t>Xcg_fuse</t>
-  </si>
-  <si>
     <t>W_wing</t>
   </si>
   <si>
-    <t>Xcg_wing</t>
-  </si>
-  <si>
     <t>W_h1</t>
   </si>
   <si>
-    <t>Xcg_h1</t>
-  </si>
-  <si>
     <t>W_h2</t>
   </si>
   <si>
-    <t>Xcg_h2</t>
-  </si>
-  <si>
     <t>W_v1</t>
   </si>
   <si>
-    <t>Xcg_v1</t>
-  </si>
-  <si>
     <t>W_v2</t>
   </si>
   <si>
-    <t>Xcg_v2</t>
-  </si>
-  <si>
     <t>W_pay</t>
   </si>
   <si>
-    <t>Xcg_pay</t>
-  </si>
-  <si>
     <t>W_ballast</t>
   </si>
   <si>
-    <t>Xcg_ballast</t>
-  </si>
-  <si>
     <t>W_systems</t>
   </si>
   <si>
-    <t>Xcg_systems</t>
-  </si>
-  <si>
-    <t>X_LE_wing</t>
-  </si>
-  <si>
-    <t>X_LE_h1</t>
-  </si>
-  <si>
-    <t>X_LE_h2</t>
-  </si>
-  <si>
-    <t>X_LE_v1</t>
-  </si>
-  <si>
-    <t>X_LE_v2</t>
-  </si>
-  <si>
     <t>Fuse_Mat</t>
   </si>
   <si>
@@ -1095,30 +1047,6 @@
     <t>rho_LWPLA</t>
   </si>
   <si>
-    <t>rho_bulk</t>
-  </si>
-  <si>
-    <t>F16</t>
-  </si>
-  <si>
-    <t>C172</t>
-  </si>
-  <si>
-    <t>B747</t>
-  </si>
-  <si>
-    <t>T38</t>
-  </si>
-  <si>
-    <t>Tiltrotor Turboprop</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>0.0082021</t>
-  </si>
-  <si>
     <t>Prop_Dia</t>
   </si>
   <si>
@@ -1210,6 +1138,33 @@
   </si>
   <si>
     <t>UAV_Prop</t>
+  </si>
+  <si>
+    <t>Bulkhead_Mat</t>
+  </si>
+  <si>
+    <t>W_wing_spar</t>
+  </si>
+  <si>
+    <t>W_bulkhead</t>
+  </si>
+  <si>
+    <t>rho_LW_balsa</t>
+  </si>
+  <si>
+    <t>N_bulkhead</t>
+  </si>
+  <si>
+    <t>Width_bulkhead</t>
+  </si>
+  <si>
+    <t>Height_bulkhead</t>
+  </si>
+  <si>
+    <t>Depth_bulkhead</t>
+  </si>
+  <si>
+    <t>0.01312 ft</t>
   </si>
 </sst>
 </file>
@@ -3291,10 +3246,10 @@
     </row>
     <row r="2" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C2" s="7">
         <v>0</v>
@@ -3483,115 +3438,115 @@
         <v>109</v>
       </c>
       <c r="E1" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="F1" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="G1" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="H1" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="I1" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="J1" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="K1" s="21" t="s">
         <v>183</v>
       </c>
-      <c r="K1" s="21" t="s">
+      <c r="L1" s="21" t="s">
         <v>184</v>
       </c>
-      <c r="L1" s="21" t="s">
+      <c r="M1" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="M1" s="21" t="s">
+      <c r="N1" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="N1" s="21" t="s">
+      <c r="O1" s="21" t="s">
         <v>187</v>
       </c>
-      <c r="O1" s="21" t="s">
+      <c r="P1" s="21" t="s">
         <v>188</v>
       </c>
-      <c r="P1" s="21" t="s">
+      <c r="Q1" s="21" t="s">
         <v>189</v>
       </c>
-      <c r="Q1" s="21" t="s">
+      <c r="R1" s="21" t="s">
         <v>190</v>
       </c>
-      <c r="R1" s="21" t="s">
+      <c r="S1" s="21" t="s">
         <v>191</v>
       </c>
-      <c r="S1" s="21" t="s">
+      <c r="T1" s="21" t="s">
         <v>192</v>
       </c>
-      <c r="T1" s="21" t="s">
+      <c r="U1" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="U1" s="21" t="s">
+      <c r="V1" s="21" t="s">
         <v>194</v>
-      </c>
-      <c r="V1" s="21" t="s">
-        <v>195</v>
       </c>
       <c r="W1" s="21" t="s">
         <v>113</v>
       </c>
       <c r="X1" s="21" t="s">
+        <v>195</v>
+      </c>
+      <c r="Y1" s="21" t="s">
         <v>196</v>
       </c>
-      <c r="Y1" s="21" t="s">
+      <c r="Z1" s="21" t="s">
         <v>197</v>
       </c>
-      <c r="Z1" s="21" t="s">
+      <c r="AA1" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="AA1" s="21" t="s">
+      <c r="AB1" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="AB1" s="21" t="s">
+      <c r="AC1" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="AC1" s="21" t="s">
+      <c r="AD1" s="21" t="s">
         <v>201</v>
       </c>
-      <c r="AD1" s="21" t="s">
+      <c r="AE1" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="AE1" s="21" t="s">
+      <c r="AF1" s="21" t="s">
         <v>203</v>
       </c>
-      <c r="AF1" s="21" t="s">
+      <c r="AG1" s="21" t="s">
         <v>204</v>
       </c>
-      <c r="AG1" s="21" t="s">
+      <c r="AH1" s="21" t="s">
         <v>205</v>
       </c>
-      <c r="AH1" s="21" t="s">
+      <c r="AI1" s="21" t="s">
         <v>206</v>
       </c>
-      <c r="AI1" s="21" t="s">
+      <c r="AJ1" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="AJ1" s="21" t="s">
+      <c r="AK1" s="21" t="s">
         <v>208</v>
       </c>
-      <c r="AK1" s="21" t="s">
+      <c r="AL1" s="21" t="s">
         <v>209</v>
       </c>
-      <c r="AL1" s="21" t="s">
+      <c r="AM1" s="21" t="s">
         <v>210</v>
       </c>
-      <c r="AM1" s="21" t="s">
+      <c r="AN1" s="21" t="s">
         <v>211</v>
       </c>
-      <c r="AN1" s="21" t="s">
+      <c r="AO1" s="21" t="s">
         <v>212</v>
-      </c>
-      <c r="AO1" s="21" t="s">
-        <v>213</v>
       </c>
       <c r="AP1" s="21" t="s">
         <v>117</v>
@@ -3635,10 +3590,10 @@
     </row>
     <row r="2" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C2" s="20">
         <v>0.14000000000000001</v>
@@ -3761,7 +3716,7 @@
         <v>1.7520000000000001E-2</v>
       </c>
       <c r="AQ2" s="20" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="AR2" s="20">
         <v>0.21</v>
@@ -3779,7 +3734,7 @@
         <v>0</v>
       </c>
       <c r="AW2" s="20" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="AX2" s="20">
         <v>0.1</v>
@@ -3807,483 +3762,215 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:AN8"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="33" width="16" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A1" s="22" t="s">
         <v>103</v>
       </c>
       <c r="B1" s="22" t="s">
+        <v>216</v>
+      </c>
+      <c r="C1" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="D1" s="22" t="s">
         <v>218</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="E1" s="22" t="s">
         <v>219</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="F1" s="22" t="s">
         <v>220</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="G1" s="22" t="s">
         <v>221</v>
       </c>
-      <c r="G1" s="22" t="s">
+      <c r="H1" s="22" t="s">
         <v>222</v>
       </c>
-      <c r="H1" s="22" t="s">
+      <c r="I1" s="22" t="s">
         <v>223</v>
       </c>
-      <c r="I1" s="22" t="s">
+      <c r="J1" s="22" t="s">
         <v>224</v>
       </c>
-      <c r="J1" s="22" t="s">
+      <c r="K1" s="22" t="s">
         <v>225</v>
       </c>
-      <c r="K1" s="22" t="s">
+      <c r="L1" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="L1" s="22" t="s">
+      <c r="M1" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="M1" s="22" t="s">
+      <c r="N1" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="N1" s="22" t="s">
+      <c r="O1" s="22" t="s">
         <v>229</v>
       </c>
-      <c r="O1" s="22" t="s">
+      <c r="P1" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="P1" s="22" t="s">
+      <c r="Q1" s="22" t="s">
         <v>231</v>
       </c>
-      <c r="Q1" s="22" t="s">
+      <c r="R1" s="22" t="s">
         <v>232</v>
       </c>
-      <c r="R1" s="22" t="s">
+      <c r="S1" s="22" t="s">
         <v>233</v>
       </c>
-      <c r="S1" s="22" t="s">
-        <v>234</v>
-      </c>
       <c r="T1" s="22" t="s">
-        <v>235</v>
+        <v>265</v>
       </c>
       <c r="U1" s="22" t="s">
-        <v>236</v>
+        <v>169</v>
       </c>
       <c r="V1" s="22" t="s">
-        <v>237</v>
+        <v>171</v>
       </c>
       <c r="W1" s="22" t="s">
-        <v>238</v>
+        <v>172</v>
       </c>
       <c r="X1" s="22" t="s">
-        <v>239</v>
+        <v>173</v>
       </c>
       <c r="Y1" s="22" t="s">
-        <v>240</v>
+        <v>174</v>
       </c>
       <c r="Z1" s="22" t="s">
-        <v>241</v>
+        <v>266</v>
       </c>
       <c r="AA1" s="22" t="s">
-        <v>242</v>
+        <v>267</v>
       </c>
       <c r="AB1" s="22" t="s">
-        <v>243</v>
+        <v>268</v>
       </c>
       <c r="AC1" s="22" t="s">
-        <v>244</v>
+        <v>269</v>
       </c>
       <c r="AD1" s="22" t="s">
-        <v>245</v>
+        <v>270</v>
       </c>
       <c r="AE1" s="22" t="s">
-        <v>246</v>
+        <v>271</v>
       </c>
       <c r="AF1" s="22" t="s">
-        <v>247</v>
-      </c>
-      <c r="AG1" s="22" t="s">
-        <v>248</v>
-      </c>
-      <c r="AH1" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="AI1" s="22" t="s">
-        <v>250</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>169</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>171</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>172</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>173</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.2">
+        <v>272</v>
+      </c>
+      <c r="AG1" s="22" t="inlineStr">
+        <is>
+          <t>N_wing_spar</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
-        <v>251</v>
-      </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
-      <c r="S2" s="22"/>
-      <c r="T2" s="22"/>
-      <c r="U2" s="22"/>
-      <c r="V2" s="22"/>
-      <c r="W2" s="22"/>
-      <c r="X2" s="22"/>
-      <c r="Y2" s="22"/>
-      <c r="Z2" s="22"/>
-      <c r="AA2" s="22"/>
-      <c r="AB2" s="22"/>
-      <c r="AC2" s="22"/>
-      <c r="AD2" s="22"/>
-      <c r="AE2" s="22"/>
-      <c r="AF2" s="22"/>
-      <c r="AG2" s="22"/>
-      <c r="AH2" s="22"/>
-      <c r="AI2" s="22"/>
-    </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.2">
-      <c r="A3" s="22" t="s">
-        <v>252</v>
-      </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
-      <c r="Y3" s="22"/>
-      <c r="Z3" s="22"/>
-      <c r="AA3" s="22"/>
-      <c r="AB3" s="22"/>
-      <c r="AC3" s="22"/>
-      <c r="AD3" s="22"/>
-      <c r="AE3" s="22"/>
-      <c r="AF3" s="22"/>
-      <c r="AG3" s="22"/>
-      <c r="AH3" s="22"/>
-      <c r="AI3" s="22"/>
-    </row>
-    <row r="4" spans="1:40" x14ac:dyDescent="0.2">
-      <c r="A4" s="22" t="s">
-        <v>253</v>
-      </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22"/>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="22"/>
-      <c r="S4" s="22"/>
-      <c r="T4" s="22"/>
-      <c r="U4" s="22"/>
-      <c r="V4" s="22"/>
-      <c r="W4" s="22"/>
-      <c r="X4" s="22"/>
-      <c r="Y4" s="22"/>
-      <c r="Z4" s="22"/>
-      <c r="AA4" s="22"/>
-      <c r="AB4" s="22"/>
-      <c r="AC4" s="22"/>
-      <c r="AD4" s="22"/>
-      <c r="AE4" s="22"/>
-      <c r="AF4" s="22"/>
-      <c r="AG4" s="22"/>
-      <c r="AH4" s="22"/>
-      <c r="AI4" s="22"/>
-    </row>
-    <row r="5" spans="1:40" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
-        <v>254</v>
-      </c>
-      <c r="B5" s="22"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="22"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="22"/>
-      <c r="V5" s="22"/>
-      <c r="W5" s="22"/>
-      <c r="X5" s="22"/>
-      <c r="Y5" s="22"/>
-      <c r="Z5" s="22"/>
-      <c r="AA5" s="22"/>
-      <c r="AB5" s="22"/>
-      <c r="AC5" s="22"/>
-      <c r="AD5" s="22"/>
-      <c r="AE5" s="22"/>
-      <c r="AF5" s="22"/>
-      <c r="AG5" s="22"/>
-      <c r="AH5" s="22"/>
-      <c r="AI5" s="22"/>
-    </row>
-    <row r="6" spans="1:40" x14ac:dyDescent="0.2">
-      <c r="A6" s="22" t="s">
-        <v>175</v>
-      </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22"/>
-      <c r="P6" s="22"/>
-      <c r="Q6" s="22"/>
-      <c r="R6" s="22"/>
-      <c r="S6" s="22"/>
-      <c r="T6" s="22"/>
-      <c r="U6" s="22"/>
-      <c r="V6" s="22"/>
-      <c r="W6" s="22"/>
-      <c r="X6" s="22"/>
-      <c r="Y6" s="22"/>
-      <c r="Z6" s="22"/>
-      <c r="AA6" s="22"/>
-      <c r="AB6" s="22"/>
-      <c r="AC6" s="22"/>
-      <c r="AD6" s="22"/>
-      <c r="AE6" s="22"/>
-      <c r="AF6" s="22"/>
-      <c r="AG6" s="22"/>
-      <c r="AH6" s="22"/>
-      <c r="AI6" s="22"/>
-    </row>
-    <row r="7" spans="1:40" x14ac:dyDescent="0.2">
-      <c r="A7" s="22" t="s">
-        <v>255</v>
-      </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22"/>
-      <c r="P7" s="22"/>
-      <c r="Q7" s="22"/>
-      <c r="R7" s="22"/>
-      <c r="S7" s="22"/>
-      <c r="T7" s="22"/>
-      <c r="U7" s="22"/>
-      <c r="V7" s="22"/>
-      <c r="W7" s="22"/>
-      <c r="X7" s="22"/>
-      <c r="Y7" s="22"/>
-      <c r="Z7" s="22"/>
-      <c r="AA7" s="22"/>
-      <c r="AB7" s="22"/>
-      <c r="AC7" s="22"/>
-      <c r="AD7" s="22"/>
-      <c r="AE7" s="22"/>
-      <c r="AF7" s="22"/>
-      <c r="AG7" s="22"/>
-      <c r="AH7" s="22"/>
-      <c r="AI7" s="22"/>
-    </row>
-    <row r="8" spans="1:40" x14ac:dyDescent="0.2">
-      <c r="A8" s="22" t="s">
-        <v>256</v>
-      </c>
-      <c r="B8" s="22">
+        <v>176</v>
+      </c>
+      <c r="B2" s="22">
         <v>0</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C2" s="22">
         <v>0</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D2" s="22">
         <v>0</v>
       </c>
-      <c r="E8" s="22">
-        <v>2.0505</v>
-      </c>
-      <c r="F8" s="22">
+      <c r="E2" s="22">
         <v>0</v>
       </c>
-      <c r="G8" s="22">
-        <v>1.2252624700000001</v>
-      </c>
-      <c r="H8" s="22">
+      <c r="F2" s="22">
         <v>0</v>
       </c>
-      <c r="I8" s="22">
-        <v>3.9</v>
-      </c>
-      <c r="J8" s="22">
+      <c r="G2" s="22">
         <v>0</v>
       </c>
-      <c r="K8" s="22">
+      <c r="H2" s="22">
         <v>0</v>
       </c>
-      <c r="L8" s="22">
+      <c r="I2" s="22">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="J2" s="22">
         <v>0</v>
       </c>
-      <c r="M8" s="22">
-        <v>3.9</v>
-      </c>
-      <c r="N8" s="22">
+      <c r="K2" s="22">
+        <v>7.4</v>
+      </c>
+      <c r="L2" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="M2" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="N2" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="O2" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="P2" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q2" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="R2" t="s">
+        <v>273</v>
+      </c>
+      <c r="S2" s="22">
+        <v>37.5</v>
+      </c>
+      <c r="T2" s="22" t="s">
+        <v>268</v>
+      </c>
+      <c r="U2" t="s">
+        <v>273</v>
+      </c>
+      <c r="V2" s="22">
+        <v>8.2021000000000004E-3</v>
+      </c>
+      <c r="W2" s="22">
+        <v>8.2021000000000004E-3</v>
+      </c>
+      <c r="X2" s="22">
+        <v>8.2021000000000004E-3</v>
+      </c>
+      <c r="Y2" s="22">
+        <v>8.2021000000000004E-3</v>
+      </c>
+      <c r="Z2" s="22">
+        <v>0.29299999999999998</v>
+      </c>
+      <c r="AA2" s="22">
         <v>0</v>
       </c>
-      <c r="O8" s="22">
-        <v>0</v>
-      </c>
-      <c r="P8" s="22">
-        <v>8.8000000000000007</v>
-      </c>
-      <c r="Q8" s="22">
-        <v>2.0299999999999998</v>
-      </c>
-      <c r="R8" s="22">
-        <v>0</v>
-      </c>
-      <c r="S8" s="22">
-        <v>0</v>
-      </c>
-      <c r="T8" s="22">
-        <v>7.4</v>
-      </c>
-      <c r="U8" s="22">
-        <v>0</v>
-      </c>
-      <c r="V8" s="22">
-        <v>1.0252624699999999</v>
-      </c>
-      <c r="W8" s="22">
-        <v>3.73</v>
-      </c>
-      <c r="X8" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y8" s="22">
-        <v>3.73</v>
-      </c>
-      <c r="Z8" s="22">
-        <v>0</v>
-      </c>
-      <c r="AA8" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="AB8" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="AC8" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="AD8" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="AE8" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="AF8" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="AG8" s="22">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="AH8" s="22">
-        <v>37.5</v>
-      </c>
-      <c r="AI8" s="22"/>
-      <c r="AJ8" t="s">
-        <v>257</v>
-      </c>
-      <c r="AK8" t="s">
-        <v>257</v>
-      </c>
-      <c r="AL8" t="s">
-        <v>257</v>
-      </c>
-      <c r="AM8" t="s">
-        <v>257</v>
-      </c>
-      <c r="AN8" t="s">
-        <v>257</v>
+      <c r="AB2" s="22">
+        <v>5.5</v>
+      </c>
+      <c r="AC2" s="22">
+        <v>4</v>
+      </c>
+      <c r="AD2" s="22">
+        <v>0.3</v>
+      </c>
+      <c r="AE2" s="22">
+        <v>0.35</v>
+      </c>
+      <c r="AF2" s="22">
+        <v>0.01</v>
+      </c>
+      <c r="AG2" s="22">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4344,33 +4031,33 @@
         <v>166</v>
       </c>
       <c r="L1" s="25" t="s">
-        <v>258</v>
+        <v>234</v>
       </c>
       <c r="M1" s="26" t="s">
-        <v>259</v>
+        <v>235</v>
       </c>
       <c r="N1" s="26" t="s">
-        <v>260</v>
+        <v>236</v>
       </c>
       <c r="O1" s="26" t="s">
-        <v>261</v>
+        <v>237</v>
       </c>
       <c r="P1" s="26" t="s">
-        <v>262</v>
+        <v>238</v>
       </c>
       <c r="Q1" s="26" t="s">
-        <v>263</v>
+        <v>239</v>
       </c>
       <c r="R1" s="26" t="s">
-        <v>264</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B2" t="s">
-        <v>265</v>
+        <v>241</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -4424,7 +4111,7 @@
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="I3" t="s">
-        <v>266</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -4453,110 +4140,110 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>267</v>
+        <v>243</v>
       </c>
       <c r="B2" t="s">
-        <v>268</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>265</v>
+        <v>241</v>
       </c>
       <c r="B3" t="s">
-        <v>269</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>270</v>
+        <v>246</v>
       </c>
       <c r="B4" t="s">
-        <v>271</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>272</v>
+        <v>248</v>
       </c>
       <c r="B5" t="s">
-        <v>273</v>
+        <v>249</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>274</v>
+        <v>250</v>
       </c>
       <c r="B6" t="s">
-        <v>275</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>276</v>
+        <v>252</v>
       </c>
       <c r="B7" t="s">
-        <v>277</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B8" s="27" t="s">
-        <v>278</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>279</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B10" s="27" t="s">
-        <v>280</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>281</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B12" s="27" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>282</v>
+        <v>258</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>283</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>284</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>285</v>
+        <v>261</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>286</v>
+        <v>262</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>287</v>
+        <v>263</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>288</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>